<commit_message>
Update Romantique SSOT copy
</commit_message>
<xml_diff>
--- a/igignore/2026-02_app_upload_확정_2/2026-02__로망띠끄__SSOT - 복사본.xlsx
+++ b/igignore/2026-02_app_upload_확정_2/2026-02__로망띠끄__SSOT - 복사본.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\limjk\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wjjo\Desktop\mapping-novel\igignore\2026-02_app_upload_확정_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F229CCB-2484-418D-AF9B-A3BA55AE322D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31470" yWindow="435" windowWidth="27465" windowHeight="15285" xr2:uid="{1C8B4D30-9719-4BA7-99BD-08E71F769C3F}"/>
+    <workbookView xWindow="31470" yWindow="435" windowWidth="27465" windowHeight="15285"/>
   </bookViews>
   <sheets>
     <sheet name="styleB(바로북)1772498411" sheetId="2" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="170">
   <si>
     <t>&gt;</t>
   </si>
@@ -28,9 +27,6 @@
     <t>styleB(바로북)   2026년 2월 1일 부터 ~ 2026년 2월 28일 까지</t>
   </si>
   <si>
-    <t>1 / 전체(1)</t>
-  </si>
-  <si>
     <t>도서코드</t>
   </si>
   <si>
@@ -67,9 +63,6 @@
     <t>판매처</t>
   </si>
   <si>
-    <t>isbn</t>
-  </si>
-  <si>
     <t>br2934</t>
   </si>
   <si>
@@ -88,36 +81,24 @@
     <t>로망띠끄</t>
   </si>
   <si>
-    <t>979-11-7530-703-2</t>
-  </si>
-  <si>
     <t>br2933</t>
   </si>
   <si>
     <t>헌터 외 사망 금지 3권</t>
   </si>
   <si>
-    <t>979-11-7530-702-5</t>
-  </si>
-  <si>
     <t>br2932</t>
   </si>
   <si>
     <t>헌터 외 사망 금지 2권</t>
   </si>
   <si>
-    <t>979-11-7530-701-8</t>
-  </si>
-  <si>
     <t>br2931</t>
   </si>
   <si>
     <t>헌터 외 사망 금지 1권</t>
   </si>
   <si>
-    <t>979-11-7530-700-1</t>
-  </si>
-  <si>
     <t>br2917</t>
   </si>
   <si>
@@ -130,9 +111,6 @@
     <t>주여명</t>
   </si>
   <si>
-    <t>979-11-7378-666-2</t>
-  </si>
-  <si>
     <t>br2916</t>
   </si>
   <si>
@@ -142,9 +120,6 @@
     <t>배이플</t>
   </si>
   <si>
-    <t>979-11-7530-665-3</t>
-  </si>
-  <si>
     <t>br2911</t>
   </si>
   <si>
@@ -157,54 +132,36 @@
     <t>아르곤18</t>
   </si>
   <si>
-    <t>979-11-7530-982-1</t>
-  </si>
-  <si>
     <t>br2910</t>
   </si>
   <si>
     <t>레드 코너 메리지 5권</t>
   </si>
   <si>
-    <t>979-11-7530-981-4</t>
-  </si>
-  <si>
     <t>br2909</t>
   </si>
   <si>
     <t>레드 코너 메리지 4권</t>
   </si>
   <si>
-    <t>979-11-7530-980-7</t>
-  </si>
-  <si>
     <t>br2908</t>
   </si>
   <si>
     <t>레드 코너 메리지 3권</t>
   </si>
   <si>
-    <t>979-11-7530-979-1</t>
-  </si>
-  <si>
     <t>br2907</t>
   </si>
   <si>
     <t>레드 코너 메리지 2권</t>
   </si>
   <si>
-    <t>979-11-7530-978-4</t>
-  </si>
-  <si>
     <t>br2906</t>
   </si>
   <si>
     <t>레드 코너 메리지 1권</t>
   </si>
   <si>
-    <t>979-11-7530-977-7</t>
-  </si>
-  <si>
     <t>br2902</t>
   </si>
   <si>
@@ -220,18 +177,12 @@
     <t>01월</t>
   </si>
   <si>
-    <t>979-11-7530-686-8</t>
-  </si>
-  <si>
     <t>br2901</t>
   </si>
   <si>
     <t>남편을 버리는 완벽한 방법 2권</t>
   </si>
   <si>
-    <t>979-11-7530-685-1</t>
-  </si>
-  <si>
     <t>br2900</t>
   </si>
   <si>
@@ -241,9 +192,6 @@
     <t>남편을 버리는 완벽한 방법 1권</t>
   </si>
   <si>
-    <t>979-11-7530-684-4</t>
-  </si>
-  <si>
     <t>br2898</t>
   </si>
   <si>
@@ -253,27 +201,18 @@
     <t>나리타</t>
   </si>
   <si>
-    <t>979-11-7530-518-2</t>
-  </si>
-  <si>
     <t>br2897</t>
   </si>
   <si>
     <t>겨울 숲의 아르덴 3권</t>
   </si>
   <si>
-    <t>979-11-7530-517-5</t>
-  </si>
-  <si>
     <t>br2896</t>
   </si>
   <si>
     <t>겨울 숲의 아르덴 2권</t>
   </si>
   <si>
-    <t>979-11-7530-516-8</t>
-  </si>
-  <si>
     <t>br2894</t>
   </si>
   <si>
@@ -283,36 +222,24 @@
     <t>유니네오</t>
   </si>
   <si>
-    <t>979-11-7530-286-0</t>
-  </si>
-  <si>
     <t>br2893</t>
   </si>
   <si>
     <t>엉덩이가 예뻐서 3권</t>
   </si>
   <si>
-    <t>979-11-7530-285-3</t>
-  </si>
-  <si>
     <t>br2892</t>
   </si>
   <si>
     <t>엉덩이가 예뻐서 2권</t>
   </si>
   <si>
-    <t>979-11-7530-284-6</t>
-  </si>
-  <si>
     <t>br2891</t>
   </si>
   <si>
     <t>엉덩이가 예뻐서 1권</t>
   </si>
   <si>
-    <t>979-11-7530-277-8</t>
-  </si>
-  <si>
     <t>br2890</t>
   </si>
   <si>
@@ -322,27 +249,18 @@
     <t>뷰이뷰이</t>
   </si>
   <si>
-    <t>979-11-7530-718-6</t>
-  </si>
-  <si>
     <t>br2889</t>
   </si>
   <si>
     <t>강아지 목에 방울 달기 2권</t>
   </si>
   <si>
-    <t>979-11-7530-717-9</t>
-  </si>
-  <si>
     <t>br2888</t>
   </si>
   <si>
     <t>강아지 목에 방울 달기 1권</t>
   </si>
   <si>
-    <t>979-11-7530-716-2</t>
-  </si>
-  <si>
     <t>br2845</t>
   </si>
   <si>
@@ -355,9 +273,6 @@
     <t>12월</t>
   </si>
   <si>
-    <t>979-11-7378-826-0</t>
-  </si>
-  <si>
     <t>br2831</t>
   </si>
   <si>
@@ -370,18 +285,12 @@
     <t>11월</t>
   </si>
   <si>
-    <t>979-11-7530-433-8</t>
-  </si>
-  <si>
     <t>br2830</t>
   </si>
   <si>
     <t>성녀가 천직이었습니다 1권</t>
   </si>
   <si>
-    <t>979-11-7530-432-1</t>
-  </si>
-  <si>
     <t>br2794</t>
   </si>
   <si>
@@ -394,45 +303,30 @@
     <t>09월</t>
   </si>
   <si>
-    <t>9791173788444</t>
-  </si>
-  <si>
     <t>br2793</t>
   </si>
   <si>
     <t>자격 없는 낮 4권</t>
   </si>
   <si>
-    <t>9791173788451</t>
-  </si>
-  <si>
     <t>br2792</t>
   </si>
   <si>
     <t>자격 없는 낮 3권</t>
   </si>
   <si>
-    <t>9791173788420</t>
-  </si>
-  <si>
     <t>br2791</t>
   </si>
   <si>
     <t>자격 없는 낮 2권</t>
   </si>
   <si>
-    <t>9791173788291</t>
-  </si>
-  <si>
     <t>br2790</t>
   </si>
   <si>
     <t>자격 없는 낮 1권</t>
   </si>
   <si>
-    <t>9791173788390</t>
-  </si>
-  <si>
     <t>br2786</t>
   </si>
   <si>
@@ -445,9 +339,6 @@
     <t>연죄</t>
   </si>
   <si>
-    <t>9791173788581</t>
-  </si>
-  <si>
     <t>br2780</t>
   </si>
   <si>
@@ -460,36 +351,24 @@
     <t>08월</t>
   </si>
   <si>
-    <t>9791173784644</t>
-  </si>
-  <si>
     <t>br2779</t>
   </si>
   <si>
     <t>궁지에 몰린 쥐는 앙하고 문다 3권</t>
   </si>
   <si>
-    <t>9791173784637</t>
-  </si>
-  <si>
     <t>br2778</t>
   </si>
   <si>
     <t>궁지에 몰린 쥐는 앙하고 문다 2권</t>
   </si>
   <si>
-    <t>9791173784620</t>
-  </si>
-  <si>
     <t>br2777</t>
   </si>
   <si>
     <t>궁지에 몰린 쥐는 앙하고 문다 1권</t>
   </si>
   <si>
-    <t>9791173784613</t>
-  </si>
-  <si>
     <t>br2723</t>
   </si>
   <si>
@@ -502,27 +381,18 @@
     <t>06월</t>
   </si>
   <si>
-    <t>9791173783609</t>
-  </si>
-  <si>
     <t>br2722</t>
   </si>
   <si>
     <t>금단의 선 2권</t>
   </si>
   <si>
-    <t>9791173783593</t>
-  </si>
-  <si>
     <t>br2721</t>
   </si>
   <si>
     <t>금단의 선 1권</t>
   </si>
   <si>
-    <t>9791173783586</t>
-  </si>
-  <si>
     <t>br2678</t>
   </si>
   <si>
@@ -535,9 +405,6 @@
     <t>05월</t>
   </si>
   <si>
-    <t>9791173782367</t>
-  </si>
-  <si>
     <t>br2602</t>
   </si>
   <si>
@@ -550,9 +417,6 @@
     <t>계바비</t>
   </si>
   <si>
-    <t>9791172924348</t>
-  </si>
-  <si>
     <t>br2551</t>
   </si>
   <si>
@@ -562,18 +426,12 @@
     <t>10월</t>
   </si>
   <si>
-    <t>9791136968227</t>
-  </si>
-  <si>
     <t>br2548</t>
   </si>
   <si>
     <t>당신을 사랑하지 않기로 했다 1권</t>
   </si>
   <si>
-    <t>9791136959584</t>
-  </si>
-  <si>
     <t>br2544</t>
   </si>
   <si>
@@ -583,90 +441,60 @@
     <t>고요(꽃잎이톡톡)</t>
   </si>
   <si>
-    <t>9791172921194</t>
-  </si>
-  <si>
     <t>br2351</t>
   </si>
   <si>
     <t>신부 수업을 1년 동안 받았습니다 1권</t>
   </si>
   <si>
-    <t>9791136943057</t>
-  </si>
-  <si>
     <t>br2266</t>
   </si>
   <si>
     <t>사소한 꽃잎 1권</t>
   </si>
   <si>
-    <t>9791136937902</t>
-  </si>
-  <si>
     <t>br2109</t>
   </si>
   <si>
     <t>이름을 세 번 부를 때까지</t>
   </si>
   <si>
-    <t>9791136925237</t>
-  </si>
-  <si>
     <t>br2107</t>
   </si>
   <si>
     <t>논 마라나타(non marana tha) 4권 (완결)</t>
   </si>
   <si>
-    <t>9791136925220</t>
-  </si>
-  <si>
     <t>br2106</t>
   </si>
   <si>
     <t>논 마라나타(non marana tha) 3권</t>
   </si>
   <si>
-    <t>9791136925213</t>
-  </si>
-  <si>
     <t>br2105</t>
   </si>
   <si>
     <t>논 마라나타(non marana tha) 2권</t>
   </si>
   <si>
-    <t>9791136925206</t>
-  </si>
-  <si>
     <t>br2104</t>
   </si>
   <si>
     <t>논 마라나타(non marana tha) 1권</t>
   </si>
   <si>
-    <t>9791136925190</t>
-  </si>
-  <si>
     <t>br2093</t>
   </si>
   <si>
     <t>서방님을 놓아드리겠습니다</t>
   </si>
   <si>
-    <t>9791136923721</t>
-  </si>
-  <si>
     <t>br1857</t>
   </si>
   <si>
     <t>곧추선 그대 (외전)</t>
   </si>
   <si>
-    <t>9791136907967</t>
-  </si>
-  <si>
     <t>br1774</t>
   </si>
   <si>
@@ -679,49 +507,34 @@
     <t>04월</t>
   </si>
   <si>
-    <t>9791133188895</t>
-  </si>
-  <si>
     <t>br1773</t>
   </si>
   <si>
     <t>흐느끼는 춘야 (외전)</t>
   </si>
   <si>
-    <t>9791133198375</t>
-  </si>
-  <si>
     <t>br1772</t>
   </si>
   <si>
     <t>흐느끼는 춘야</t>
   </si>
   <si>
-    <t>9791133196425</t>
-  </si>
-  <si>
     <t>br1769</t>
   </si>
   <si>
     <t>냉궁마마</t>
   </si>
   <si>
-    <t>9791133198887</t>
-  </si>
-  <si>
     <t>br1741</t>
   </si>
   <si>
     <t>곧추선 그대</t>
-  </si>
-  <si>
-    <t>9791133199297</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1114,7 +927,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -1328,43 +1141,6 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
       <right/>
       <top style="thin">
         <color rgb="FF000000"/>
@@ -1527,7 +1303,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1606,22 +1382,13 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1998,8 +1765,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5086BCA4-5B33-4DC1-9F4B-65951CE5AF7B}">
-  <dimension ref="A1:M67"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L67"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5" customWidth="1"/>
@@ -2013,10 +1780,9 @@
     <col min="10" max="10" width="15.5" customWidth="1"/>
     <col min="11" max="11" width="12.25" customWidth="1"/>
     <col min="12" max="12" width="16.125" customWidth="1"/>
-    <col min="13" max="13" width="18.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -2031,11 +1797,8 @@
       <c r="J1" s="15"/>
       <c r="K1" s="15"/>
       <c r="L1" s="16"/>
-      <c r="M1" s="26" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17"/>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
@@ -2048,9 +1811,8 @@
       <c r="J2" s="18"/>
       <c r="K2" s="18"/>
       <c r="L2" s="19"/>
-      <c r="M2" s="27"/>
-    </row>
-    <row r="3" spans="1:13" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
         <v>1</v>
       </c>
@@ -2065,9 +1827,8 @@
       <c r="J3" s="21"/>
       <c r="K3" s="21"/>
       <c r="L3" s="22"/>
-      <c r="M3" s="27"/>
-    </row>
-    <row r="4" spans="1:13" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:12" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
@@ -2080,63 +1841,59 @@
       <c r="J4" s="24"/>
       <c r="K4" s="24"/>
       <c r="L4" s="25"/>
-      <c r="M4" s="28"/>
-    </row>
-    <row r="5" spans="1:13" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:12" s="2" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="3" t="s">
+    </row>
+    <row r="6" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>16</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>17</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>19</v>
       </c>
       <c r="G6" s="7">
         <v>1</v>
@@ -2151,29 +1908,26 @@
         <v>1815</v>
       </c>
       <c r="K6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>20</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>23</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G7" s="7">
         <v>1</v>
@@ -2188,29 +1942,26 @@
         <v>1815</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G8" s="7">
         <v>1</v>
@@ -2225,29 +1976,26 @@
         <v>1815</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G9" s="7">
         <v>1</v>
@@ -2262,29 +2010,26 @@
         <v>1815</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G10" s="7">
         <v>1</v>
@@ -2299,29 +2044,26 @@
         <v>1870</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M10" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" s="4" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" s="4" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="G11" s="7">
         <v>1</v>
@@ -2336,29 +2078,26 @@
         <v>1815</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G12" s="7">
         <v>1</v>
@@ -2373,29 +2112,26 @@
         <v>1925</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G13" s="7">
         <v>1</v>
@@ -2410,29 +2146,26 @@
         <v>1925</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M13" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G14" s="7">
         <v>1</v>
@@ -2447,29 +2180,26 @@
         <v>1925</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M14" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G15" s="7">
         <v>1</v>
@@ -2484,29 +2214,26 @@
         <v>1925</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G16" s="7">
         <v>1</v>
@@ -2521,29 +2248,26 @@
         <v>1925</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G17" s="7">
         <v>1</v>
@@ -2558,29 +2282,26 @@
         <v>1925</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M17" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G18" s="7">
         <v>3</v>
@@ -2595,29 +2316,26 @@
         <v>4950</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G19" s="7">
         <v>1</v>
@@ -2632,29 +2350,26 @@
         <v>1650</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G20" s="7">
         <v>3</v>
@@ -2669,29 +2384,26 @@
         <v>4950</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M20" s="6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="G21" s="7">
         <v>6</v>
@@ -2706,29 +2418,26 @@
         <v>9900</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M21" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G22" s="7">
         <v>1</v>
@@ -2743,29 +2452,26 @@
         <v>1760</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M22" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G23" s="7">
         <v>1</v>
@@ -2780,29 +2486,26 @@
         <v>1760</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M23" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G24" s="7">
         <v>1</v>
@@ -2817,29 +2520,26 @@
         <v>1760</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M24" s="6" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="G25" s="7">
         <v>2</v>
@@ -2854,29 +2554,26 @@
         <v>3300</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M25" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5" t="s">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="G26" s="7">
         <v>2</v>
@@ -2891,29 +2588,26 @@
         <v>3300</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M26" s="6" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="5"/>
       <c r="D27" s="5" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="G27" s="7">
         <v>2</v>
@@ -2928,29 +2622,26 @@
         <v>3300</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M27" s="6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="5"/>
       <c r="D28" s="5" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="G28" s="7">
         <v>3</v>
@@ -2965,29 +2656,26 @@
         <v>4950</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M28" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="G29" s="7">
         <v>1</v>
@@ -3002,29 +2690,26 @@
         <v>1760</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M29" s="6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="5"/>
       <c r="D30" s="5" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="G30" s="7">
         <v>1</v>
@@ -3039,29 +2724,26 @@
         <v>1760</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M30" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="5"/>
       <c r="D31" s="5" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="G31" s="7">
         <v>1</v>
@@ -3076,29 +2758,26 @@
         <v>1760</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M31" s="6" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="5"/>
       <c r="D32" s="5" t="s">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>109</v>
+        <v>82</v>
       </c>
       <c r="G32" s="7">
         <v>3</v>
@@ -3113,29 +2792,26 @@
         <v>4950</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M32" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>114</v>
+        <v>86</v>
       </c>
       <c r="G33" s="7">
         <v>1</v>
@@ -3150,29 +2826,26 @@
         <v>1650</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M33" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="5"/>
       <c r="D34" s="5" t="s">
-        <v>118</v>
+        <v>89</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>114</v>
+        <v>86</v>
       </c>
       <c r="G34" s="7">
         <v>1</v>
@@ -3187,29 +2860,26 @@
         <v>1650</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M34" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="G35" s="7">
         <v>1</v>
@@ -3224,29 +2894,26 @@
         <v>880</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M35" s="6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>125</v>
+        <v>94</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="5"/>
       <c r="D36" s="5" t="s">
-        <v>126</v>
+        <v>95</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="G36" s="7">
         <v>1</v>
@@ -3261,29 +2928,26 @@
         <v>1815</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M36" s="6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="5"/>
       <c r="D37" s="5" t="s">
-        <v>129</v>
+        <v>97</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="G37" s="7">
         <v>1</v>
@@ -3298,29 +2962,26 @@
         <v>1815</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M37" s="6" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>131</v>
+        <v>98</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>132</v>
+        <v>99</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="G38" s="7">
         <v>1</v>
@@ -3335,29 +2996,26 @@
         <v>1815</v>
       </c>
       <c r="K38" s="7" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M38" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>134</v>
+        <v>100</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>135</v>
+        <v>101</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="G39" s="7">
         <v>1</v>
@@ -3372,29 +3030,26 @@
         <v>1815</v>
       </c>
       <c r="K39" s="7" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="L39" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M39" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>137</v>
+        <v>102</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>138</v>
+        <v>103</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>139</v>
+        <v>104</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>140</v>
+        <v>105</v>
       </c>
       <c r="G40" s="7">
         <v>1</v>
@@ -3409,29 +3064,26 @@
         <v>660</v>
       </c>
       <c r="K40" s="7" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="L40" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M40" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>142</v>
+        <v>106</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>143</v>
+        <v>107</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="G41" s="7">
         <v>1</v>
@@ -3446,29 +3098,26 @@
         <v>1815</v>
       </c>
       <c r="K41" s="7" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="L41" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M41" s="6" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>147</v>
+        <v>110</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>148</v>
+        <v>111</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="G42" s="7">
         <v>1</v>
@@ -3483,29 +3132,26 @@
         <v>1815</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="L42" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M42" s="6" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>150</v>
+        <v>112</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>151</v>
+        <v>113</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="G43" s="7">
         <v>1</v>
@@ -3520,29 +3166,26 @@
         <v>1815</v>
       </c>
       <c r="K43" s="7" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="L43" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M43" s="6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>153</v>
+        <v>114</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>154</v>
+        <v>115</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="G44" s="7">
         <v>1</v>
@@ -3557,29 +3200,26 @@
         <v>1815</v>
       </c>
       <c r="K44" s="7" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="L44" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M44" s="6" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>156</v>
+        <v>116</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>157</v>
+        <v>117</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>158</v>
+        <v>118</v>
       </c>
       <c r="G45" s="7">
         <v>1</v>
@@ -3594,29 +3234,26 @@
         <v>1760</v>
       </c>
       <c r="K45" s="7" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="L45" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M45" s="6" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>161</v>
+        <v>120</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>162</v>
+        <v>121</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>158</v>
+        <v>118</v>
       </c>
       <c r="G46" s="7">
         <v>1</v>
@@ -3631,29 +3268,26 @@
         <v>1760</v>
       </c>
       <c r="K46" s="7" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="L46" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M46" s="6" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>164</v>
+        <v>122</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="5"/>
       <c r="D47" s="5" t="s">
-        <v>165</v>
+        <v>123</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>158</v>
+        <v>118</v>
       </c>
       <c r="G47" s="7">
         <v>1</v>
@@ -3668,29 +3302,26 @@
         <v>1760</v>
       </c>
       <c r="K47" s="7" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="L47" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M47" s="6" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>167</v>
+        <v>124</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
-        <v>168</v>
+        <v>125</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>169</v>
+        <v>126</v>
       </c>
       <c r="G48" s="7">
         <v>1</v>
@@ -3705,29 +3336,26 @@
         <v>825</v>
       </c>
       <c r="K48" s="7" t="s">
-        <v>170</v>
+        <v>127</v>
       </c>
       <c r="L48" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M48" s="6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>172</v>
+        <v>128</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>173</v>
+        <v>129</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>174</v>
+        <v>130</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>175</v>
+        <v>131</v>
       </c>
       <c r="G49" s="7">
         <v>1</v>
@@ -3742,29 +3370,26 @@
         <v>1650</v>
       </c>
       <c r="K49" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="L49" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M49" s="6" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>177</v>
+        <v>132</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>178</v>
+        <v>133</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="G50" s="7">
         <v>1</v>
@@ -3779,29 +3404,26 @@
         <v>1980</v>
       </c>
       <c r="K50" s="7" t="s">
-        <v>179</v>
+        <v>134</v>
       </c>
       <c r="L50" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M50" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>181</v>
+        <v>135</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="5"/>
       <c r="D51" s="5" t="s">
-        <v>182</v>
+        <v>136</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="G51" s="7">
         <v>1</v>
@@ -3816,29 +3438,26 @@
         <v>1980</v>
       </c>
       <c r="K51" s="7" t="s">
-        <v>179</v>
+        <v>134</v>
       </c>
       <c r="L51" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M51" s="6" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>184</v>
+        <v>137</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>185</v>
+        <v>138</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F52" s="7" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="G52" s="7">
         <v>1</v>
@@ -3853,29 +3472,26 @@
         <v>1980</v>
       </c>
       <c r="K52" s="7" t="s">
-        <v>179</v>
+        <v>134</v>
       </c>
       <c r="L52" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M52" s="6" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>188</v>
+        <v>140</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>189</v>
+        <v>141</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G53" s="7">
         <v>1</v>
@@ -3890,29 +3506,26 @@
         <v>1760</v>
       </c>
       <c r="K53" s="7" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L53" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M53" s="6" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="54" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>191</v>
+        <v>142</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>192</v>
+        <v>143</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G54" s="7">
         <v>1</v>
@@ -3927,29 +3540,26 @@
         <v>1925</v>
       </c>
       <c r="K54" s="7" t="s">
-        <v>170</v>
+        <v>127</v>
       </c>
       <c r="L54" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M54" s="6" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>194</v>
+        <v>144</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>195</v>
+        <v>145</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>169</v>
+        <v>126</v>
       </c>
       <c r="G55" s="7">
         <v>1</v>
@@ -3964,29 +3574,26 @@
         <v>2200</v>
       </c>
       <c r="K55" s="7" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="L55" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M55" s="6" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="56" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
-        <v>197</v>
+        <v>146</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>198</v>
+        <v>147</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>169</v>
+        <v>126</v>
       </c>
       <c r="G56" s="7">
         <v>1</v>
@@ -4001,29 +3608,26 @@
         <v>2255</v>
       </c>
       <c r="K56" s="7" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="L56" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M56" s="6" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="57" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
-        <v>200</v>
+        <v>148</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>201</v>
+        <v>149</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>169</v>
+        <v>126</v>
       </c>
       <c r="G57" s="7">
         <v>1</v>
@@ -4038,29 +3642,26 @@
         <v>2090</v>
       </c>
       <c r="K57" s="7" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="L57" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M57" s="6" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="58" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
-        <v>203</v>
+        <v>150</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>204</v>
+        <v>151</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>169</v>
+        <v>126</v>
       </c>
       <c r="G58" s="7">
         <v>1</v>
@@ -4075,29 +3676,26 @@
         <v>2035</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="L58" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M58" s="6" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="59" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>206</v>
+        <v>152</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="5"/>
       <c r="D59" s="5" t="s">
-        <v>207</v>
+        <v>153</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>169</v>
+        <v>126</v>
       </c>
       <c r="G59" s="7">
         <v>1</v>
@@ -4112,29 +3710,26 @@
         <v>2035</v>
       </c>
       <c r="K59" s="7" t="s">
-        <v>159</v>
+        <v>119</v>
       </c>
       <c r="L59" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M59" s="6" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="60" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>209</v>
+        <v>154</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="5"/>
       <c r="D60" s="5" t="s">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="G60" s="7">
         <v>2</v>
@@ -4149,29 +3744,26 @@
         <v>3850</v>
       </c>
       <c r="K60" s="7" t="s">
-        <v>170</v>
+        <v>127</v>
       </c>
       <c r="L60" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M60" s="6" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="61" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
-        <v>212</v>
+        <v>156</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="5"/>
       <c r="D61" s="5" t="s">
-        <v>213</v>
+        <v>157</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="G61" s="7">
         <v>3</v>
@@ -4186,29 +3778,26 @@
         <v>495</v>
       </c>
       <c r="K61" s="7" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
       <c r="L61" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M61" s="6" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="62" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>215</v>
+        <v>158</v>
       </c>
       <c r="B62" s="6"/>
       <c r="C62" s="5"/>
       <c r="D62" s="5" t="s">
-        <v>216</v>
+        <v>159</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="G62" s="7">
         <v>2</v>
@@ -4223,29 +3812,26 @@
         <v>1650</v>
       </c>
       <c r="K62" s="7" t="s">
-        <v>218</v>
+        <v>161</v>
       </c>
       <c r="L62" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M62" s="6" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="63" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>220</v>
+        <v>162</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="5"/>
       <c r="D63" s="5" t="s">
-        <v>221</v>
+        <v>163</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="G63" s="7">
         <v>1</v>
@@ -4260,29 +3846,26 @@
         <v>165</v>
       </c>
       <c r="K63" s="7" t="s">
-        <v>218</v>
+        <v>161</v>
       </c>
       <c r="L63" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M63" s="6" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="64" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
-        <v>223</v>
+        <v>164</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="5"/>
       <c r="D64" s="5" t="s">
-        <v>224</v>
+        <v>165</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="G64" s="7">
         <v>2</v>
@@ -4297,29 +3880,26 @@
         <v>3850</v>
       </c>
       <c r="K64" s="7" t="s">
-        <v>218</v>
+        <v>161</v>
       </c>
       <c r="L64" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M64" s="6" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="65" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
-        <v>226</v>
+        <v>166</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" s="5"/>
       <c r="D65" s="5" t="s">
-        <v>227</v>
+        <v>167</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="G65" s="7">
         <v>2</v>
@@ -4334,29 +3914,26 @@
         <v>3520</v>
       </c>
       <c r="K65" s="7" t="s">
-        <v>218</v>
+        <v>161</v>
       </c>
       <c r="L65" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M65" s="6" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="66" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
-        <v>229</v>
+        <v>168</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="5"/>
       <c r="D66" s="5" t="s">
-        <v>230</v>
+        <v>169</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="G66" s="7">
         <v>3</v>
@@ -4371,22 +3948,19 @@
         <v>4950</v>
       </c>
       <c r="K66" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="L66" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M66" s="6" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="67" spans="1:13" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="29"/>
-      <c r="B67" s="30"/>
-      <c r="C67" s="30"/>
-      <c r="D67" s="30"/>
-      <c r="E67" s="30"/>
-      <c r="F67" s="31"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="26"/>
+      <c r="B67" s="27"/>
+      <c r="C67" s="27"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="27"/>
+      <c r="F67" s="28"/>
       <c r="G67" s="5">
         <v>85</v>
       </c>
@@ -4399,16 +3973,14 @@
       </c>
       <c r="K67" s="5"/>
       <c r="L67" s="5"/>
-      <c r="M67" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
+    <mergeCell ref="A67:F67"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="A4:L4"/>
-    <mergeCell ref="M1:M4"/>
-    <mergeCell ref="A67:F67"/>
   </mergeCells>
   <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>